<commit_message>
wip(tests): r3/r4/e2e follow the dataset EV-2 story; regenerate orders_seed.xlsx (#20)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ANcWPGENfoWFq5LV8cUSBX
</commit_message>
<xml_diff>
--- a/data/orders_seed.xlsx
+++ b/data/orders_seed.xlsx
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -652,7 +652,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -3416,17 +3416,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>J-CURE-07-10021614</t>
+          <t>J-CURE-07-10021150</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>#M-201</t>
+          <t>#S-101</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3436,16 +3436,16 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>MD-M201</t>
+          <t>MD-S101</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-10-02T16:14:00+08:00</t>
+          <t>2026-10-02T11:50:00+08:00</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
@@ -3568,17 +3568,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>J-CURE-11-10021012</t>
+          <t>J-CURE-11-10021612</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>#S-101</t>
+          <t>#M-201</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -3588,16 +3588,16 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MD-S101</t>
+          <t>MD-M201</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-10-02T10:12:00+08:00</t>
+          <t>2026-10-02T16:12:00+08:00</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H12" t="n">
         <v>1</v>
@@ -4012,69 +4012,69 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-02T15:40:00+08:00</t>
+          <t>2026-10-02T11:50:00+08:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>A-MIX</t>
+          <t>CURE-07</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>QC 取樣</t>
+          <t>入模</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>qc</t>
+          <t>curing</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>CURI-早2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>#L-301</t>
+          <t>#S-101</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>門尼黏度 62，合格</t>
+          <t>小胎入模，128°C，預計 24 h</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-02T16:14:00+08:00</t>
+          <t>2026-10-02T15:40:00+08:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CURE-07</t>
+          <t>A-MIX</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>入模</t>
+          <t>QC 取樣</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>curing</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>CURI-中1</t>
+          <t>qc</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>#M-201</t>
+          <t>#L-301</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>中胎入模，128°C，預計 28 h</t>
+          <t>門尼黏度 62，合格</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs+tests: dataset order book is the sim's order book; regenerate orders_seed.xlsx (#20 第 1 題)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ANcWPGENfoWFq5LV8cUSBX
</commit_message>
<xml_diff>
--- a/data/orders_seed.xlsx
+++ b/data/orders_seed.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>#S-101</t>
+          <t>SO-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -476,10 +476,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="D2" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -488,12 +488,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>南亞堆高機</t>
+          <t>客戶A</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>MD-S101</t>
+          <t>MD-SO-001</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -503,33 +503,33 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>#S-102</t>
+          <t>SO-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>台灣搬運車</t>
+          <t>客戶B</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>MD-S102</t>
+          <t>MD-SO-002</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -539,33 +539,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>#M-201</t>
+          <t>SO-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>高雄港機具</t>
+          <t>客戶C</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>MD-M201</t>
+          <t>MD-SO-003</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -575,33 +575,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>#M-202</t>
+          <t>SO-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-11-17</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>東元物流</t>
+          <t>客戶D</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>MD-M202</t>
+          <t>MD-SO-004</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -611,33 +611,33 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>#L-301</t>
+          <t>SO-005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-12-24</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>台中港務</t>
+          <t>客戶D</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>MD-L301</t>
+          <t>MD-SO-005</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -647,7 +647,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>#A-311</t>
+          <t>SO-006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -656,34 +656,34 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>台塑工業車輛</t>
+          <t>客戶E</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>#A-311</t>
+          <t>MD-SO-006</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>#L-302</t>
+          <t>SO-007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -692,28 +692,136 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>41</v>
+        <v>80</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-12-02</t>
+          <t>2027-01-03</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>中鋼運輸</t>
+          <t>客戶E</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>MD-L302</t>
+          <t>MD-SO-007</t>
         </is>
       </c>
       <c r="H8" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SO-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>客戶F</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>MD-SO-008</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SO-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>客戶G</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>MD-SO-009</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>#A-311</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>台塑工業車輛</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>#A-311</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -3140,7 +3248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3188,12 +3296,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>J-CURE-01-10030012</t>
+          <t>J-CURE-03-10020320</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>#S-101</t>
+          <t>SO-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3203,17 +3311,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CURE-01</t>
+          <t>CURE-03</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>MD-S101</t>
+          <t>MD-SO-001</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-10-03T00:12:00+08:00</t>
+          <t>2026-10-02T03:20:00+08:00</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -3226,12 +3334,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>J-CURE-02-10022012</t>
+          <t>J-CURE-04-10020430</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>#S-101</t>
+          <t>SO-001</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3241,17 +3349,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CURE-02</t>
+          <t>CURE-04</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MD-S101</t>
+          <t>MD-SO-001</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-10-02T20:12:00+08:00</t>
+          <t>2026-10-02T04:30:00+08:00</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -3264,12 +3372,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>J-CURE-03-10021612</t>
+          <t>J-CURE-05-10020910</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>#S-101</t>
+          <t>SO-001</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3279,17 +3387,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CURE-03</t>
+          <t>CURE-05</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>MD-S101</t>
+          <t>MD-SO-001</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-10-02T16:12:00+08:00</t>
+          <t>2026-10-02T09:10:00+08:00</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -3302,12 +3410,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>J-CURE-04-10021212</t>
+          <t>J-CURE-06-10021040</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>#S-101</t>
+          <t>SO-001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3317,17 +3425,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CURE-04</t>
+          <t>CURE-06</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>MD-S101</t>
+          <t>MD-SO-001</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-10-02T12:12:00+08:00</t>
+          <t>2026-10-02T10:40:00+08:00</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -3340,12 +3448,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>J-CURE-05-10020812</t>
+          <t>J-CURE-07-10021150</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>#S-101</t>
+          <t>SO-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3355,17 +3463,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CURE-05</t>
+          <t>CURE-07</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>MD-S101</t>
+          <t>MD-SO-001</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-10-02T08:12:00+08:00</t>
+          <t>2026-10-02T11:50:00+08:00</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -3378,36 +3486,36 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>J-CURE-06-10020512</t>
+          <t>J-CURE-08-10021630</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>#S-101</t>
+          <t>SO-002</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CURE-06</t>
+          <t>CURE-08</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>MD-S101</t>
+          <t>MD-SO-002</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-10-02T05:12:00+08:00</t>
+          <t>2026-10-02T16:30:00+08:00</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H7" t="n">
         <v>1</v>
@@ -3416,36 +3524,36 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>J-CURE-07-10021150</t>
+          <t>J-CURE-09-10022130</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>#S-101</t>
+          <t>SO-002</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CURE-07</t>
+          <t>CURE-09</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>MD-S101</t>
+          <t>MD-SO-002</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-10-02T11:50:00+08:00</t>
+          <t>2026-10-02T21:30:00+08:00</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
@@ -3454,12 +3562,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>J-CURE-08-10020612</t>
+          <t>J-CURE-11-10012200</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>#L-301</t>
+          <t>SO-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3469,137 +3577,23 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CURE-08</t>
+          <t>CURE-11</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MD-L301</t>
+          <t>MD-SO-003</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-10-02T06:12:00+08:00</t>
+          <t>2026-10-01T22:00:00+08:00</t>
         </is>
       </c>
       <c r="G9" t="n">
         <v>34</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>J-CURE-09-10020212</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>#M-201</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>CURE-09</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>MD-M201</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026-10-02T02:12:00+08:00</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>28</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>J-CURE-10-10022012</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>#L-301</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>CURE-10</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>MD-L301</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2026-10-02T20:12:00+08:00</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>34</v>
-      </c>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>J-CURE-11-10021612</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>#M-201</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>CURE-11</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>MD-M201</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2026-10-02T16:12:00+08:00</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>28</v>
-      </c>
-      <c r="H12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3906,49 +3900,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-02T02:12:00+08:00</t>
+          <t>2026-10-02T10:05:00+08:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CURE-09</t>
+          <t>A-BIGOPEN</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>入模</t>
+          <t>巡檢</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>body</t>
+          <t>bigopen</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BODY-夜1</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>#M-201</t>
+          <t>BIGO-早1</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>中胎入模，128°C，預計 28 h</t>
+          <t>膠溫 96°C，水流正常</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-02T06:12:00+08:00</t>
+          <t>2026-10-02T11:50:00+08:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CURE-08</t>
+          <t>CURE-07</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3968,56 +3957,56 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>#L-301</t>
+          <t>SO-001</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>大胎入模，128°C，預計 34 h</t>
+          <t>小胎入模，128°C，預計 24 h</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-02T10:05:00+08:00</t>
+          <t>2026-10-02T15:40:00+08:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A-BIGOPEN</t>
+          <t>A-MIX</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>巡檢</t>
+          <t>QC 取樣</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>bigopen</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>BIGO-早1</t>
+          <t>qc</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>#L-301</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>膠溫 96°C，水流正常</t>
+          <t>門尼黏度 62，合格</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-02T11:50:00+08:00</t>
+          <t>2026-10-02T16:30:00+08:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CURE-07</t>
+          <t>CURE-08</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4032,88 +4021,93 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CURI-早2</t>
+          <t>CURI-中1</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>#S-101</t>
+          <t>SO-002</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>小胎入模，128°C，預計 24 h</t>
+          <t>中胎入模，128°C，預計 28 h</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-02T15:40:00+08:00</t>
+          <t>2026-10-02T18:00:00+08:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>A-MIX</t>
+          <t>CURE-03</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>QC 取樣</t>
+          <t>保養</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>qc</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>#L-301</t>
+          <t>maintenance</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>門尼黏度 62，合格</t>
+          <t>更換疏水閥墊片</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-02T18:00:00+08:00</t>
+          <t>2026-10-02T20:12:00+08:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CURE-03</t>
+          <t>CURE-10</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>保養</t>
+          <t>入模</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>maintenance</t>
+          <t>body</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BODY-夜1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>#L-301</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>更換疏水閥墊片</t>
+          <t>大胎入模，128°C，預計 34 h</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-02T20:12:00+08:00</t>
+          <t>2026-10-02T21:30:00+08:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CURE-10</t>
+          <t>CURE-09</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4133,12 +4127,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>#L-301</t>
+          <t>SO-002</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>大胎入模，128°C，預計 34 h</t>
+          <t>中胎入模，128°C，預計 28 h</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: replace placeholder customer names with fictional Taiwanese-style companies
Replaces 客戶A–G (team dataset) and 客戶甲～癸 (simulator) with 17 invented
company names, using one fixed mapping (recorded in data/team_dataset/README.md).
The two sets stay separate customers. #A-311 in orders_seed.xlsx (台塑工業車輛)
now matches the dataset (永固機械股份有限公司).

Only names changed: order ids, sizes, quantities, due dates and all other
workbook cells/formulas are identical to before. No agent, scheduler or tool
logic touched. warroom/kb/orders_db.py seed names, bench/results, data/runtime
and databases are intentionally left unchanged.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011PbDzaQixnScn2P8vt6nwK
</commit_message>
<xml_diff>
--- a/data/orders_seed.xlsx
+++ b/data/orders_seed.xlsx
@@ -488,7 +488,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>客戶A</t>
+          <t>福氣輪業股份有限公司</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -524,7 +524,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>客戶B</t>
+          <t>金旺來工業社</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>客戶C</t>
+          <t>大力出奇蹟實業有限公司</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>客戶D</t>
+          <t>永固機械股份有限公司</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>客戶D</t>
+          <t>永固機械股份有限公司</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>客戶E</t>
+          <t>黑狗兄輪業商社</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>客戶E</t>
+          <t>黑狗兄輪業商社</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>客戶F</t>
+          <t>好運輪輪來企業社</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>客戶G</t>
+          <t>鐵牛運搬股份有限公司</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>台塑工業車輛</t>
+          <t>永固機械股份有限公司</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>